<commit_message>
Usable money first: read K2 Sum of Usable, show runway in bal, stats, digest and dashboard
- lib/usable: parse K2 SUM of C cells into usable accounts (fallback: all but Savings)
- bal/stats/Sunday digest lead with usable total and days it lasts at the 30-day average
- dashboard: Usable now card with runway and usable-over-time line; balances split usable / not usable
- template: K2 Sum of Usable (Savings excluded)
</commit_message>
<xml_diff>
--- a/template/Budget_Template.xlsx
+++ b/template/Budget_Template.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="49">
   <si>
     <t>Balance</t>
   </si>
@@ -23,6 +23,9 @@
   </si>
   <si>
     <t>Start</t>
+  </si>
+  <si>
+    <t>Sum of Usable</t>
   </si>
   <si>
     <t>Category</t>
@@ -571,17 +574,20 @@
       <c r="H1" s="1">
         <f>TEXT(DATE($R$1,($R$2-1)*3+3,1),"mmmm")</f>
       </c>
+      <c r="K1" s="1" t="s">
+        <v>3</v>
+      </c>
       <c r="P1" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R1">
         <v>2026</v>
       </c>
       <c r="S1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="3:19" x14ac:dyDescent="0.25">
@@ -603,8 +609,11 @@
       <c r="H2">
         <f>IF($D2="","",SUMIFS(E$20:E$901,$A$20:$A$901,"&gt;="&amp;DATE($R$1,($R$2-1)*3+3,1),$A$20:$A$901,"&lt;"&amp;IF($R$2=4,DATE($R$1+1,1,1),DATE($R$1,$R$2*3+1,1))))</f>
       </c>
+      <c r="K2">
+        <f>SUM(C2,C3,C4)</f>
+      </c>
       <c r="P2" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q2">
         <f>IF(P2="","",-(SUMIFS(E$20:E$901,$C$20:$C$901,P2,$B$20:$B$901,"Expense")+SUMIFS(F$20:F$901,$C$20:$C$901,P2,$B$20:$B$901,"Expense")+SUMIFS(G$20:G$901,$C$20:$C$901,P2,$B$20:$B$901,"Expense")+SUMIFS(H$20:H$901,$C$20:$C$901,P2,$B$20:$B$901,"Expense")+SUMIFS(I$20:I$901,$C$20:$C$901,P2,$B$20:$B$901,"Expense")+SUMIFS(J$20:J$901,$C$20:$C$901,P2,$B$20:$B$901,"Expense")+SUMIFS(K$20:K$901,$C$20:$C$901,P2,$B$20:$B$901,"Expense")+SUMIFS(L$20:L$901,$C$20:$C$901,P2,$B$20:$B$901,"Expense")+SUMIFS(M$20:M$901,$C$20:$C$901,P2,$B$20:$B$901,"Expense")+SUMIFS(N$20:N$901,$C$20:$C$901,P2,$B$20:$B$901,"Expense")))</f>
@@ -613,7 +622,7 @@
         <v>4</v>
       </c>
       <c r="S2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="3:17" x14ac:dyDescent="0.25">
@@ -636,7 +645,7 @@
         <f>IF($D3="","",SUMIFS(F$20:F$901,$A$20:$A$901,"&gt;="&amp;DATE($R$1,($R$2-1)*3+3,1),$A$20:$A$901,"&lt;"&amp;IF($R$2=4,DATE($R$1+1,1,1),DATE($R$1,$R$2*3+1,1))))</f>
       </c>
       <c r="P3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q3">
         <f>IF(P3="","",-(SUMIFS(E$20:E$901,$C$20:$C$901,P3,$B$20:$B$901,"Expense")+SUMIFS(F$20:F$901,$C$20:$C$901,P3,$B$20:$B$901,"Expense")+SUMIFS(G$20:G$901,$C$20:$C$901,P3,$B$20:$B$901,"Expense")+SUMIFS(H$20:H$901,$C$20:$C$901,P3,$B$20:$B$901,"Expense")+SUMIFS(I$20:I$901,$C$20:$C$901,P3,$B$20:$B$901,"Expense")+SUMIFS(J$20:J$901,$C$20:$C$901,P3,$B$20:$B$901,"Expense")+SUMIFS(K$20:K$901,$C$20:$C$901,P3,$B$20:$B$901,"Expense")+SUMIFS(L$20:L$901,$C$20:$C$901,P3,$B$20:$B$901,"Expense")+SUMIFS(M$20:M$901,$C$20:$C$901,P3,$B$20:$B$901,"Expense")+SUMIFS(N$20:N$901,$C$20:$C$901,P3,$B$20:$B$901,"Expense")))</f>
@@ -662,7 +671,7 @@
         <f>IF($D4="","",SUMIFS(G$20:G$901,$A$20:$A$901,"&gt;="&amp;DATE($R$1,($R$2-1)*3+3,1),$A$20:$A$901,"&lt;"&amp;IF($R$2=4,DATE($R$1+1,1,1),DATE($R$1,$R$2*3+1,1))))</f>
       </c>
       <c r="P4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q4">
         <f>IF(P4="","",-(SUMIFS(E$20:E$901,$C$20:$C$901,P4,$B$20:$B$901,"Expense")+SUMIFS(F$20:F$901,$C$20:$C$901,P4,$B$20:$B$901,"Expense")+SUMIFS(G$20:G$901,$C$20:$C$901,P4,$B$20:$B$901,"Expense")+SUMIFS(H$20:H$901,$C$20:$C$901,P4,$B$20:$B$901,"Expense")+SUMIFS(I$20:I$901,$C$20:$C$901,P4,$B$20:$B$901,"Expense")+SUMIFS(J$20:J$901,$C$20:$C$901,P4,$B$20:$B$901,"Expense")+SUMIFS(K$20:K$901,$C$20:$C$901,P4,$B$20:$B$901,"Expense")+SUMIFS(L$20:L$901,$C$20:$C$901,P4,$B$20:$B$901,"Expense")+SUMIFS(M$20:M$901,$C$20:$C$901,P4,$B$20:$B$901,"Expense")+SUMIFS(N$20:N$901,$C$20:$C$901,P4,$B$20:$B$901,"Expense")))</f>
@@ -688,7 +697,7 @@
         <f>IF($D5="","",SUMIFS(H$20:H$901,$A$20:$A$901,"&gt;="&amp;DATE($R$1,($R$2-1)*3+3,1),$A$20:$A$901,"&lt;"&amp;IF($R$2=4,DATE($R$1+1,1,1),DATE($R$1,$R$2*3+1,1))))</f>
       </c>
       <c r="P5" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q5">
         <f>IF(P5="","",-(SUMIFS(E$20:E$901,$C$20:$C$901,P5,$B$20:$B$901,"Expense")+SUMIFS(F$20:F$901,$C$20:$C$901,P5,$B$20:$B$901,"Expense")+SUMIFS(G$20:G$901,$C$20:$C$901,P5,$B$20:$B$901,"Expense")+SUMIFS(H$20:H$901,$C$20:$C$901,P5,$B$20:$B$901,"Expense")+SUMIFS(I$20:I$901,$C$20:$C$901,P5,$B$20:$B$901,"Expense")+SUMIFS(J$20:J$901,$C$20:$C$901,P5,$B$20:$B$901,"Expense")+SUMIFS(K$20:K$901,$C$20:$C$901,P5,$B$20:$B$901,"Expense")+SUMIFS(L$20:L$901,$C$20:$C$901,P5,$B$20:$B$901,"Expense")+SUMIFS(M$20:M$901,$C$20:$C$901,P5,$B$20:$B$901,"Expense")+SUMIFS(N$20:N$901,$C$20:$C$901,P5,$B$20:$B$901,"Expense")))</f>
@@ -714,7 +723,7 @@
         <f>IF($D6="","",SUMIFS(I$20:I$901,$A$20:$A$901,"&gt;="&amp;DATE($R$1,($R$2-1)*3+3,1),$A$20:$A$901,"&lt;"&amp;IF($R$2=4,DATE($R$1+1,1,1),DATE($R$1,$R$2*3+1,1))))</f>
       </c>
       <c r="P6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q6">
         <f>IF(P6="","",-(SUMIFS(E$20:E$901,$C$20:$C$901,P6,$B$20:$B$901,"Expense")+SUMIFS(F$20:F$901,$C$20:$C$901,P6,$B$20:$B$901,"Expense")+SUMIFS(G$20:G$901,$C$20:$C$901,P6,$B$20:$B$901,"Expense")+SUMIFS(H$20:H$901,$C$20:$C$901,P6,$B$20:$B$901,"Expense")+SUMIFS(I$20:I$901,$C$20:$C$901,P6,$B$20:$B$901,"Expense")+SUMIFS(J$20:J$901,$C$20:$C$901,P6,$B$20:$B$901,"Expense")+SUMIFS(K$20:K$901,$C$20:$C$901,P6,$B$20:$B$901,"Expense")+SUMIFS(L$20:L$901,$C$20:$C$901,P6,$B$20:$B$901,"Expense")+SUMIFS(M$20:M$901,$C$20:$C$901,P6,$B$20:$B$901,"Expense")+SUMIFS(N$20:N$901,$C$20:$C$901,P6,$B$20:$B$901,"Expense")))</f>
@@ -740,7 +749,7 @@
         <f>IF($D7="","",SUMIFS(J$20:J$901,$A$20:$A$901,"&gt;="&amp;DATE($R$1,($R$2-1)*3+3,1),$A$20:$A$901,"&lt;"&amp;IF($R$2=4,DATE($R$1+1,1,1),DATE($R$1,$R$2*3+1,1))))</f>
       </c>
       <c r="P7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q7">
         <f>IF(P7="","",-(SUMIFS(E$20:E$901,$C$20:$C$901,P7,$B$20:$B$901,"Expense")+SUMIFS(F$20:F$901,$C$20:$C$901,P7,$B$20:$B$901,"Expense")+SUMIFS(G$20:G$901,$C$20:$C$901,P7,$B$20:$B$901,"Expense")+SUMIFS(H$20:H$901,$C$20:$C$901,P7,$B$20:$B$901,"Expense")+SUMIFS(I$20:I$901,$C$20:$C$901,P7,$B$20:$B$901,"Expense")+SUMIFS(J$20:J$901,$C$20:$C$901,P7,$B$20:$B$901,"Expense")+SUMIFS(K$20:K$901,$C$20:$C$901,P7,$B$20:$B$901,"Expense")+SUMIFS(L$20:L$901,$C$20:$C$901,P7,$B$20:$B$901,"Expense")+SUMIFS(M$20:M$901,$C$20:$C$901,P7,$B$20:$B$901,"Expense")+SUMIFS(N$20:N$901,$C$20:$C$901,P7,$B$20:$B$901,"Expense")))</f>
@@ -766,7 +775,7 @@
         <f>IF($D8="","",SUMIFS(K$20:K$901,$A$20:$A$901,"&gt;="&amp;DATE($R$1,($R$2-1)*3+3,1),$A$20:$A$901,"&lt;"&amp;IF($R$2=4,DATE($R$1+1,1,1),DATE($R$1,$R$2*3+1,1))))</f>
       </c>
       <c r="P8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q8">
         <f>IF(P8="","",-(SUMIFS(E$20:E$901,$C$20:$C$901,P8,$B$20:$B$901,"Expense")+SUMIFS(F$20:F$901,$C$20:$C$901,P8,$B$20:$B$901,"Expense")+SUMIFS(G$20:G$901,$C$20:$C$901,P8,$B$20:$B$901,"Expense")+SUMIFS(H$20:H$901,$C$20:$C$901,P8,$B$20:$B$901,"Expense")+SUMIFS(I$20:I$901,$C$20:$C$901,P8,$B$20:$B$901,"Expense")+SUMIFS(J$20:J$901,$C$20:$C$901,P8,$B$20:$B$901,"Expense")+SUMIFS(K$20:K$901,$C$20:$C$901,P8,$B$20:$B$901,"Expense")+SUMIFS(L$20:L$901,$C$20:$C$901,P8,$B$20:$B$901,"Expense")+SUMIFS(M$20:M$901,$C$20:$C$901,P8,$B$20:$B$901,"Expense")+SUMIFS(N$20:N$901,$C$20:$C$901,P8,$B$20:$B$901,"Expense")))</f>
@@ -792,7 +801,7 @@
         <f>IF($D9="","",SUMIFS(L$20:L$901,$A$20:$A$901,"&gt;="&amp;DATE($R$1,($R$2-1)*3+3,1),$A$20:$A$901,"&lt;"&amp;IF($R$2=4,DATE($R$1+1,1,1),DATE($R$1,$R$2*3+1,1))))</f>
       </c>
       <c r="P9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q9">
         <f>IF(P9="","",-(SUMIFS(E$20:E$901,$C$20:$C$901,P9,$B$20:$B$901,"Expense")+SUMIFS(F$20:F$901,$C$20:$C$901,P9,$B$20:$B$901,"Expense")+SUMIFS(G$20:G$901,$C$20:$C$901,P9,$B$20:$B$901,"Expense")+SUMIFS(H$20:H$901,$C$20:$C$901,P9,$B$20:$B$901,"Expense")+SUMIFS(I$20:I$901,$C$20:$C$901,P9,$B$20:$B$901,"Expense")+SUMIFS(J$20:J$901,$C$20:$C$901,P9,$B$20:$B$901,"Expense")+SUMIFS(K$20:K$901,$C$20:$C$901,P9,$B$20:$B$901,"Expense")+SUMIFS(L$20:L$901,$C$20:$C$901,P9,$B$20:$B$901,"Expense")+SUMIFS(M$20:M$901,$C$20:$C$901,P9,$B$20:$B$901,"Expense")+SUMIFS(N$20:N$901,$C$20:$C$901,P9,$B$20:$B$901,"Expense")))</f>
@@ -818,7 +827,7 @@
         <f>IF($D10="","",SUMIFS(M$20:M$901,$A$20:$A$901,"&gt;="&amp;DATE($R$1,($R$2-1)*3+3,1),$A$20:$A$901,"&lt;"&amp;IF($R$2=4,DATE($R$1+1,1,1),DATE($R$1,$R$2*3+1,1))))</f>
       </c>
       <c r="P10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q10">
         <f>IF(P10="","",-(SUMIFS(E$20:E$901,$C$20:$C$901,P10,$B$20:$B$901,"Expense")+SUMIFS(F$20:F$901,$C$20:$C$901,P10,$B$20:$B$901,"Expense")+SUMIFS(G$20:G$901,$C$20:$C$901,P10,$B$20:$B$901,"Expense")+SUMIFS(H$20:H$901,$C$20:$C$901,P10,$B$20:$B$901,"Expense")+SUMIFS(I$20:I$901,$C$20:$C$901,P10,$B$20:$B$901,"Expense")+SUMIFS(J$20:J$901,$C$20:$C$901,P10,$B$20:$B$901,"Expense")+SUMIFS(K$20:K$901,$C$20:$C$901,P10,$B$20:$B$901,"Expense")+SUMIFS(L$20:L$901,$C$20:$C$901,P10,$B$20:$B$901,"Expense")+SUMIFS(M$20:M$901,$C$20:$C$901,P10,$B$20:$B$901,"Expense")+SUMIFS(N$20:N$901,$C$20:$C$901,P10,$B$20:$B$901,"Expense")))</f>
@@ -844,7 +853,7 @@
         <f>IF($D11="","",SUMIFS(N$20:N$901,$A$20:$A$901,"&gt;="&amp;DATE($R$1,($R$2-1)*3+3,1),$A$20:$A$901,"&lt;"&amp;IF($R$2=4,DATE($R$1+1,1,1),DATE($R$1,$R$2*3+1,1))))</f>
       </c>
       <c r="P11" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q11">
         <f>IF(P11="","",-(SUMIFS(E$20:E$901,$C$20:$C$901,P11,$B$20:$B$901,"Expense")+SUMIFS(F$20:F$901,$C$20:$C$901,P11,$B$20:$B$901,"Expense")+SUMIFS(G$20:G$901,$C$20:$C$901,P11,$B$20:$B$901,"Expense")+SUMIFS(H$20:H$901,$C$20:$C$901,P11,$B$20:$B$901,"Expense")+SUMIFS(I$20:I$901,$C$20:$C$901,P11,$B$20:$B$901,"Expense")+SUMIFS(J$20:J$901,$C$20:$C$901,P11,$B$20:$B$901,"Expense")+SUMIFS(K$20:K$901,$C$20:$C$901,P11,$B$20:$B$901,"Expense")+SUMIFS(L$20:L$901,$C$20:$C$901,P11,$B$20:$B$901,"Expense")+SUMIFS(M$20:M$901,$C$20:$C$901,P11,$B$20:$B$901,"Expense")+SUMIFS(N$20:N$901,$C$20:$C$901,P11,$B$20:$B$901,"Expense")))</f>
@@ -860,7 +869,7 @@
         <f>SUM(C2:C11)</f>
       </c>
       <c r="D13" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E13">
         <f>SUM(E2:E11)</f>
@@ -900,31 +909,31 @@
     </row>
     <row r="18" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O18" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="Q18" s="1">
         <f>IF(P18="","",-(SUMIFS(E$20:E$901,$C$20:$C$901,P18,$B$20:$B$901,"Expense")+SUMIFS(F$20:F$901,$C$20:$C$901,P18,$B$20:$B$901,"Expense")+SUMIFS(G$20:G$901,$C$20:$C$901,P18,$B$20:$B$901,"Expense")+SUMIFS(H$20:H$901,$C$20:$C$901,P18,$B$20:$B$901,"Expense")+SUMIFS(I$20:I$901,$C$20:$C$901,P18,$B$20:$B$901,"Expense")+SUMIFS(J$20:J$901,$C$20:$C$901,P18,$B$20:$B$901,"Expense")+SUMIFS(K$20:K$901,$C$20:$C$901,P18,$B$20:$B$901,"Expense")+SUMIFS(L$20:L$901,$C$20:$C$901,P18,$B$20:$B$901,"Expense")+SUMIFS(M$20:M$901,$C$20:$C$901,P18,$B$20:$B$901,"Expense")+SUMIFS(N$20:N$901,$C$20:$C$901,P18,$B$20:$B$901,"Expense")))</f>
@@ -3708,20 +3717,20 @@
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="2:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C6">
         <v>6000</v>
@@ -3729,7 +3738,7 @@
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7">
         <v>1000</v>
@@ -3737,7 +3746,7 @@
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C8">
         <v>1500</v>
@@ -3745,7 +3754,7 @@
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C9">
         <v>2000</v>
@@ -3753,7 +3762,7 @@
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C10">
         <v>2000</v>
@@ -3761,7 +3770,7 @@
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B11" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C11">
         <v>500</v>
@@ -3769,7 +3778,7 @@
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B12" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C12">
         <v>1000</v>
@@ -3777,7 +3786,7 @@
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B13" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C13">
         <v>1000</v>
@@ -3785,7 +3794,7 @@
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B14" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C14">
         <v>1000</v>
@@ -3793,7 +3802,7 @@
     </row>
     <row r="15" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B15" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -3812,102 +3821,102 @@
   <sheetData>
     <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -3926,37 +3935,37 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>